<commit_message>
chỉnh lại cấu trúc folder
</commit_message>
<xml_diff>
--- a/ai/data/metadata_scored_final.xlsx
+++ b/ai/data/metadata_scored_final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\NCKH\CNN_dog_cat\backend\PetAI\ai\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{452A4AEB-6662-4E4B-934C-EA47E19EA742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27DEDAD1-CBDA-44E3-8187-458A2DD136BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1487" uniqueCount="675">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1467" uniqueCount="675">
   <si>
     <t>STT</t>
   </si>
@@ -3212,8 +3212,8 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="8.88671875" style="1"/>
-    <col min="3" max="3" width="26.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="8.88671875" style="1"/>
+    <col min="3" max="3" width="26.5546875" style="1" customWidth="1"/>
+    <col min="4" max="7" width="8.88671875" style="1" customWidth="1"/>
     <col min="8" max="8" width="13.21875" style="1" customWidth="1"/>
     <col min="9" max="9" width="25.33203125" style="1" customWidth="1"/>
     <col min="10" max="10" width="19.5546875" style="1" customWidth="1"/>
@@ -10528,21 +10528,11 @@
       <c r="I142" s="4"/>
       <c r="J142" s="4"/>
       <c r="K142" s="4"/>
-      <c r="L142" s="4">
-        <v>3</v>
-      </c>
-      <c r="M142" s="4">
-        <v>3</v>
-      </c>
-      <c r="N142" s="4">
-        <v>3</v>
-      </c>
-      <c r="O142" s="4">
-        <v>3</v>
-      </c>
-      <c r="P142" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="L142" s="4"/>
+      <c r="M142" s="4"/>
+      <c r="N142" s="4"/>
+      <c r="O142" s="4"/>
+      <c r="P142" s="4"/>
       <c r="Q142" s="4"/>
     </row>
   </sheetData>

</xml_diff>